<commit_message>
Update prices from Google Sheets
</commit_message>
<xml_diff>
--- a/public/projects.xlsx
+++ b/public/projects.xlsx
@@ -13,65 +13,65 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="97">
+  <si>
+    <t>Setting</t>
+  </si>
+  <si>
+    <t>How to fill the Projects sheet</t>
+  </si>
   <si>
     <t>Project</t>
   </si>
   <si>
-    <t>How to fill the Projects sheet</t>
-  </si>
-  <si>
-    <t>Setting</t>
+    <t>Value</t>
   </si>
   <si>
     <t>Type</t>
   </si>
   <si>
+    <t>Company Name</t>
+  </si>
+  <si>
+    <t>Alahly Sabbour</t>
+  </si>
+  <si>
+    <t>BUA</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>BUA</t>
-  </si>
-  <si>
-    <t>Company Name</t>
+    <t>Currency</t>
   </si>
   <si>
     <t>Phase</t>
   </si>
   <si>
-    <t>Alahly Sabbour</t>
+    <t>EGP</t>
   </si>
   <si>
     <t>Plan</t>
   </si>
   <si>
-    <t>Currency</t>
+    <t>Each row is ONE payment plan. Rows with a blank Project cell belong to the project above them.</t>
   </si>
   <si>
     <t>Years</t>
   </si>
   <si>
-    <t>Each row is ONE payment plan. Rows with a blank Project cell belong to the project above them.</t>
-  </si>
-  <si>
-    <t>EGP</t>
-  </si>
-  <si>
     <t>Discount %</t>
   </si>
   <si>
     <t>Down Payment Type</t>
   </si>
   <si>
+    <t>كل صف = نظام سداد واحد. لو خلية المشروع فاضية، الصف بيتبع المشروع اللي فوقه.</t>
+  </si>
+  <si>
     <t>Down Payment 1 %</t>
   </si>
   <si>
-    <t>كل صف = نظام سداد واحد. لو خلية المشروع فاضية، الصف بيتبع المشروع اللي فوقه.</t>
-  </si>
-  <si>
     <t>Down Payment 2 %</t>
   </si>
   <si>
@@ -81,78 +81,78 @@
     <t>Installments Count</t>
   </si>
   <si>
+    <t>Installment Every (months)</t>
+  </si>
+  <si>
+    <t>First Installment Due (months)</t>
+  </si>
+  <si>
+    <t>Maintenance %</t>
+  </si>
+  <si>
     <t>All % columns are plain numbers in percent units: 10 means 10%, 0.99 means 0.99%.</t>
   </si>
   <si>
-    <t>Installment Every (months)</t>
-  </si>
-  <si>
     <t>أعمدة النسب أرقام عادية: 10 يعني 10%، و 0.99 يعني 0.99%.</t>
   </si>
   <si>
-    <t>First Installment Due (months)</t>
-  </si>
-  <si>
-    <t>Maintenance %</t>
+    <t>Delivery (months)</t>
   </si>
   <si>
     <t>Cells formatted as % in Excel (showing "10%") are also understood correctly.</t>
   </si>
   <si>
-    <t>Delivery (months)</t>
-  </si>
-  <si>
     <t>ولو نسّقت الخلية كنسبة مئوية في إكسل، هتتفهم صح برضه.</t>
   </si>
   <si>
     <t>First Installment Maintenance Due (months)</t>
   </si>
   <si>
+    <t>Ending Installment Maintenance Due (months)</t>
+  </si>
+  <si>
     <t>Column</t>
   </si>
   <si>
     <t>Meaning / المعنى</t>
   </si>
   <si>
-    <t>Ending Installment Maintenance Due (months)</t>
+    <t>Maintenance Basis</t>
+  </si>
+  <si>
+    <t>YOUD</t>
   </si>
   <si>
     <t>Project name. Leave blank to repeat the project above. / اسم المشروع — سيبها فاضية لتكرار اللي فوق</t>
   </si>
   <si>
-    <t>Maintenance Basis</t>
-  </si>
-  <si>
-    <t>YOUD</t>
-  </si>
-  <si>
     <t>Plan label shown in the dropdown, e.g. "8 Years" or "Cash" / اسم نظام السداد</t>
   </si>
   <si>
     <t>Plan length in years, 0 for cash (informational) / مدة النظام بالسنين</t>
   </si>
   <si>
+    <t>Discount off the system price; negative = premium / نسبة الخصم من سعر النظام</t>
+  </si>
+  <si>
+    <t>First down payment, % of selling price, due at contract date / المقدم الأول</t>
+  </si>
+  <si>
+    <t>Second down payment, 0 if none / المقدم الثاني</t>
+  </si>
+  <si>
     <t>5% DP &amp; 5% After 3 Months &amp; 8 Years</t>
   </si>
   <si>
+    <t>When DP2 is due, months after contract / استحقاق المقدم الثاني بعد كام شهر</t>
+  </si>
+  <si>
+    <t>Number of equal installments / عدد الأقساط</t>
+  </si>
+  <si>
     <t>Original Price</t>
   </si>
   <si>
-    <t>Discount off the system price; negative = premium / نسبة الخصم من سعر النظام</t>
-  </si>
-  <si>
-    <t>First down payment, % of selling price, due at contract date / المقدم الأول</t>
-  </si>
-  <si>
-    <t>Second down payment, 0 if none / المقدم الثاني</t>
-  </si>
-  <si>
-    <t>When DP2 is due, months after contract / استحقاق المقدم الثاني بعد كام شهر</t>
-  </si>
-  <si>
-    <t>Number of equal installments / عدد الأقساط</t>
-  </si>
-  <si>
     <t>3 = quarterly, 1 = monthly / الفترة بين الأقساط بالشهور</t>
   </si>
   <si>
@@ -174,21 +174,21 @@
     <t>% of system price, due at delivery / وديعة الصيانة</t>
   </si>
   <si>
+    <t>Months from contract to delivery / الاستلام بعد كام شهر</t>
+  </si>
+  <si>
+    <t>After editing: save the file, then refresh the page in the browser.</t>
+  </si>
+  <si>
+    <t>بعد التعديل: احفظ الملف واعمل refresh للصفحة.</t>
+  </si>
+  <si>
     <t>Selling price</t>
   </si>
   <si>
-    <t>Months from contract to delivery / الاستلام بعد كام شهر</t>
-  </si>
-  <si>
     <t>10% DP &amp; 8 Years</t>
   </si>
   <si>
-    <t>After editing: save the file, then refresh the page in the browser.</t>
-  </si>
-  <si>
-    <t>بعد التعديل: احفظ الملف واعمل refresh للصفحة.</t>
-  </si>
-  <si>
     <t>7.5% DP &amp; 7.5% After 3 Months &amp; 8 Years</t>
   </si>
   <si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>GAIA</t>
+  </si>
+  <si>
+    <t>SUMMER</t>
   </si>
 </sst>
 </file>
@@ -600,22 +603,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>15</v>
@@ -624,7 +627,7 @@
         <v>16</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>19</v>
@@ -636,39 +639,39 @@
         <v>21</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="O1" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>30</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F2" s="1">
         <v>8.0</v>
@@ -677,7 +680,7 @@
         <v>0.0</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I2" s="1">
         <v>5.0</v>
@@ -715,15 +718,15 @@
         <v>6.0</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F3" s="1">
         <v>8.0</v>
@@ -732,7 +735,7 @@
         <v>10.0</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I3" s="1">
         <v>10.0</v>
@@ -770,12 +773,12 @@
         <v>6.0</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>58</v>
@@ -787,7 +790,7 @@
         <v>15.0</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I4" s="1">
         <v>7.5</v>
@@ -825,12 +828,12 @@
         <v>6.0</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>59</v>
@@ -842,7 +845,7 @@
         <v>20.0</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I5" s="1">
         <v>10.0</v>
@@ -879,12 +882,12 @@
         <v>6.0</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>60</v>
@@ -896,7 +899,7 @@
         <v>25.0</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I6" s="1">
         <v>12.5</v>
@@ -933,12 +936,12 @@
         <v>6.0</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>61</v>
@@ -950,7 +953,7 @@
         <v>30.0</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I7" s="1">
         <v>15.0</v>
@@ -987,12 +990,12 @@
         <v>6.0</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>62</v>
@@ -1004,7 +1007,7 @@
         <v>35.0</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I8" s="1">
         <v>17.5</v>
@@ -1041,12 +1044,12 @@
         <v>6.0</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>63</v>
@@ -1058,7 +1061,7 @@
         <v>40.0</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I9" s="1">
         <v>20.0</v>
@@ -1095,12 +1098,12 @@
         <v>6.0</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>64</v>
@@ -1112,7 +1115,7 @@
         <v>45.0</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I10" s="1">
         <v>22.5</v>
@@ -1149,12 +1152,12 @@
         <v>6.0</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>65</v>
@@ -1169,7 +1172,7 @@
         <v>50.0</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I11" s="1">
         <v>25.0</v>
@@ -1205,12 +1208,12 @@
         <v>6.0</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D12" s="3">
         <v>4.0</v>
@@ -1225,7 +1228,7 @@
         <v>50.0</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I12" s="1">
         <v>25.0</v>
@@ -1262,7 +1265,7 @@
         <v>6.0</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -1270,7 +1273,7 @@
         <v>67</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F13" s="1">
         <v>8.0</v>
@@ -1279,7 +1282,7 @@
         <v>0.0</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I13" s="1">
         <v>5.0</v>
@@ -1317,7 +1320,7 @@
         <v>6.0</v>
       </c>
       <c r="T13" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14">
@@ -1325,7 +1328,7 @@
         <v>67</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F14" s="1">
         <v>8.0</v>
@@ -1334,7 +1337,7 @@
         <v>10.0</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I14" s="1">
         <v>10.0</v>
@@ -1372,7 +1375,7 @@
         <v>6.0</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15">
@@ -1389,7 +1392,7 @@
         <v>15.0</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I15" s="1">
         <v>7.5</v>
@@ -1427,7 +1430,7 @@
         <v>6.0</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16">
@@ -1444,7 +1447,7 @@
         <v>20.0</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I16" s="1">
         <v>10.0</v>
@@ -1482,7 +1485,7 @@
         <v>6.0</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17">
@@ -1499,7 +1502,7 @@
         <v>25.0</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I17" s="1">
         <v>12.5</v>
@@ -1537,7 +1540,7 @@
         <v>6.0</v>
       </c>
       <c r="T17" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18">
@@ -1554,7 +1557,7 @@
         <v>30.0</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I18" s="1">
         <v>15.0</v>
@@ -1592,7 +1595,7 @@
         <v>6.0</v>
       </c>
       <c r="T18" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19">
@@ -1609,7 +1612,7 @@
         <v>35.0</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I19" s="1">
         <v>17.5</v>
@@ -1647,7 +1650,7 @@
         <v>6.0</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20">
@@ -1664,7 +1667,7 @@
         <v>40.0</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I20" s="1">
         <v>20.0</v>
@@ -1702,7 +1705,7 @@
         <v>6.0</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21">
@@ -1719,7 +1722,7 @@
         <v>45.0</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I21" s="1">
         <v>22.5</v>
@@ -1757,7 +1760,7 @@
         <v>6.0</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22">
@@ -1774,7 +1777,7 @@
         <v>50.0</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I22" s="1">
         <v>25.0</v>
@@ -1812,7 +1815,7 @@
         <v>6.0</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23">
@@ -1829,7 +1832,7 @@
         <v>0.0</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I23" s="1">
         <v>10.0</v>
@@ -1865,7 +1868,7 @@
         <v>3.0</v>
       </c>
       <c r="T23" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24">
@@ -1882,7 +1885,7 @@
         <v>0.0</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I24" s="3">
         <v>15.0</v>
@@ -1918,7 +1921,7 @@
         <v>3.0</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25">
@@ -1935,7 +1938,7 @@
         <v>0.0</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I25" s="3">
         <v>20.0</v>
@@ -1971,7 +1974,7 @@
         <v>3.0</v>
       </c>
       <c r="T25" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26">
@@ -1988,7 +1991,7 @@
         <v>0.0</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I26" s="3">
         <v>25.0</v>
@@ -2024,7 +2027,7 @@
         <v>3.0</v>
       </c>
       <c r="T26" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27">
@@ -2041,7 +2044,7 @@
         <v>0.0</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I27" s="3">
         <v>30.0</v>
@@ -2077,7 +2080,7 @@
         <v>3.0</v>
       </c>
       <c r="T27" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28">
@@ -2094,7 +2097,7 @@
         <v>0.0</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I28" s="3">
         <v>35.0</v>
@@ -2130,7 +2133,7 @@
         <v>3.0</v>
       </c>
       <c r="T28" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29">
@@ -2147,7 +2150,7 @@
         <v>0.0</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I29" s="3">
         <v>40.0</v>
@@ -2183,7 +2186,7 @@
         <v>3.0</v>
       </c>
       <c r="T29" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30">
@@ -2200,7 +2203,7 @@
         <v>15.0</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I30" s="1">
         <v>100.0</v>
@@ -2236,7 +2239,7 @@
         <v>3.0</v>
       </c>
       <c r="T30" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31">
@@ -2253,7 +2256,7 @@
         <v>0.0</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I31" s="3">
         <v>10.0</v>
@@ -2290,7 +2293,7 @@
         <v>3.0</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32">
@@ -2307,7 +2310,7 @@
         <v>0.0</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I32" s="3">
         <v>15.0</v>
@@ -2343,7 +2346,7 @@
         <v>3.0</v>
       </c>
       <c r="T32" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33">
@@ -2360,7 +2363,7 @@
         <v>0.0</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I33" s="3">
         <v>20.0</v>
@@ -2396,7 +2399,7 @@
         <v>3.0</v>
       </c>
       <c r="T33" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34">
@@ -2413,7 +2416,7 @@
         <v>0.0</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I34" s="3">
         <v>25.0</v>
@@ -2449,7 +2452,7 @@
         <v>3.0</v>
       </c>
       <c r="T34" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="35">
@@ -2466,7 +2469,7 @@
         <v>0.0</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I35" s="3">
         <v>30.0</v>
@@ -2502,7 +2505,7 @@
         <v>3.0</v>
       </c>
       <c r="T35" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36">
@@ -2519,7 +2522,7 @@
         <v>0.0</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I36" s="3">
         <v>35.0</v>
@@ -2555,7 +2558,7 @@
         <v>3.0</v>
       </c>
       <c r="T36" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="37">
@@ -2572,7 +2575,7 @@
         <v>0.0</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I37" s="3">
         <v>40.0</v>
@@ -2608,7 +2611,7 @@
         <v>3.0</v>
       </c>
       <c r="T37" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38">
@@ -2625,7 +2628,7 @@
         <v>15.0</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I38" s="3">
         <v>100.0</v>
@@ -2661,7 +2664,7 @@
         <v>3.0</v>
       </c>
       <c r="T38" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="39">
@@ -2681,7 +2684,7 @@
         <v>25.0</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I39" s="1">
         <v>100.0</v>
@@ -2717,7 +2720,7 @@
         <v>6.0</v>
       </c>
       <c r="T39" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40">
@@ -2734,7 +2737,7 @@
         <v>0.0</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I40" s="1">
         <v>5.0</v>
@@ -2770,7 +2773,7 @@
         <v>6.0</v>
       </c>
       <c r="T40" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41">
@@ -2787,7 +2790,7 @@
         <v>3.0</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I41" s="1">
         <v>5.0</v>
@@ -2823,7 +2826,7 @@
         <v>6.0</v>
       </c>
       <c r="T41" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42">
@@ -2840,7 +2843,7 @@
         <v>6.0</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I42" s="1">
         <v>5.0</v>
@@ -2876,7 +2879,7 @@
         <v>6.0</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43">
@@ -2893,7 +2896,7 @@
         <v>9.0</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I43" s="1">
         <v>5.0</v>
@@ -2929,7 +2932,7 @@
         <v>6.0</v>
       </c>
       <c r="T43" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44">
@@ -2949,7 +2952,7 @@
         <v>25.0</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I44" s="1">
         <v>100.0</v>
@@ -2985,7 +2988,7 @@
         <v>6.0</v>
       </c>
       <c r="T44" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45">
@@ -3005,7 +3008,7 @@
         <v>0.0</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I45" s="1">
         <v>5.0</v>
@@ -3041,7 +3044,7 @@
         <v>6.0</v>
       </c>
       <c r="T45" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46">
@@ -3061,7 +3064,7 @@
         <v>3.0</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I46" s="1">
         <v>5.0</v>
@@ -3097,7 +3100,7 @@
         <v>6.0</v>
       </c>
       <c r="T46" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="47">
@@ -3117,7 +3120,7 @@
         <v>6.0</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I47" s="1">
         <v>5.0</v>
@@ -3153,7 +3156,7 @@
         <v>6.0</v>
       </c>
       <c r="T47" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48">
@@ -3173,7 +3176,7 @@
         <v>9.0</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I48" s="1">
         <v>5.0</v>
@@ -3209,7 +3212,7 @@
         <v>6.0</v>
       </c>
       <c r="T48" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="49">
@@ -3217,7 +3220,7 @@
         <v>93</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F49" s="1">
         <v>8.0</v>
@@ -3226,7 +3229,7 @@
         <v>0.0</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I49" s="1">
         <v>5.0</v>
@@ -3263,12 +3266,12 @@
         <v>6.0</v>
       </c>
       <c r="T49" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50">
       <c r="E50" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F50" s="1">
         <v>8.0</v>
@@ -3277,7 +3280,7 @@
         <v>10.0</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I50" s="1">
         <v>10.0</v>
@@ -3314,7 +3317,7 @@
         <v>6.0</v>
       </c>
       <c r="T50" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51">
@@ -3328,7 +3331,7 @@
         <v>15.0</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I51" s="1">
         <v>7.5</v>
@@ -3365,7 +3368,7 @@
         <v>6.0</v>
       </c>
       <c r="T51" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="52">
@@ -3379,7 +3382,7 @@
         <v>20.0</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I52" s="1">
         <v>10.0</v>
@@ -3416,7 +3419,7 @@
         <v>6.0</v>
       </c>
       <c r="T52" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="53">
@@ -3430,7 +3433,7 @@
         <v>25.0</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I53" s="1">
         <v>12.5</v>
@@ -3467,7 +3470,7 @@
         <v>6.0</v>
       </c>
       <c r="T53" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="54">
@@ -3481,7 +3484,7 @@
         <v>30.0</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I54" s="1">
         <v>15.0</v>
@@ -3518,7 +3521,7 @@
         <v>6.0</v>
       </c>
       <c r="T54" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="55">
@@ -3532,7 +3535,7 @@
         <v>35.0</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I55" s="1">
         <v>17.5</v>
@@ -3569,7 +3572,7 @@
         <v>6.0</v>
       </c>
       <c r="T55" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56">
@@ -3583,7 +3586,7 @@
         <v>40.0</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I56" s="1">
         <v>20.0</v>
@@ -3620,7 +3623,7 @@
         <v>6.0</v>
       </c>
       <c r="T56" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="57">
@@ -3634,7 +3637,7 @@
         <v>45.0</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I57" s="1">
         <v>22.5</v>
@@ -3671,7 +3674,7 @@
         <v>6.0</v>
       </c>
       <c r="T57" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="58">
@@ -3685,7 +3688,7 @@
         <v>50.0</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I58" s="1">
         <v>25.0</v>
@@ -3722,7 +3725,7 @@
         <v>6.0</v>
       </c>
       <c r="T58" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59">
@@ -3730,7 +3733,7 @@
         <v>94</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F59" s="1">
         <v>8.0</v>
@@ -3739,7 +3742,7 @@
         <v>0.0</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I59" s="1">
         <v>5.0</v>
@@ -3775,12 +3778,12 @@
         <v>3.0</v>
       </c>
       <c r="T59" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="60">
       <c r="E60" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F60" s="1">
         <v>8.0</v>
@@ -3789,7 +3792,7 @@
         <v>10.0</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I60" s="1">
         <v>10.0</v>
@@ -3825,7 +3828,7 @@
         <v>3.0</v>
       </c>
       <c r="T60" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61">
@@ -3839,7 +3842,7 @@
         <v>15.0</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I61" s="1">
         <v>7.5</v>
@@ -3875,7 +3878,7 @@
         <v>3.0</v>
       </c>
       <c r="T61" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="62">
@@ -3889,7 +3892,7 @@
         <v>20.0</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I62" s="1">
         <v>10.0</v>
@@ -3925,7 +3928,7 @@
         <v>3.0</v>
       </c>
       <c r="T62" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="63">
@@ -3939,7 +3942,7 @@
         <v>25.0</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I63" s="1">
         <v>12.5</v>
@@ -3975,7 +3978,7 @@
         <v>3.0</v>
       </c>
       <c r="T63" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="64">
@@ -3989,7 +3992,7 @@
         <v>30.0</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I64" s="1">
         <v>15.0</v>
@@ -4025,7 +4028,7 @@
         <v>3.0</v>
       </c>
       <c r="T64" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="65">
@@ -4039,7 +4042,7 @@
         <v>35.0</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I65" s="1">
         <v>17.5</v>
@@ -4075,7 +4078,7 @@
         <v>3.0</v>
       </c>
       <c r="T65" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="66">
@@ -4089,7 +4092,7 @@
         <v>40.0</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I66" s="1">
         <v>20.0</v>
@@ -4125,7 +4128,7 @@
         <v>3.0</v>
       </c>
       <c r="T66" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="67">
@@ -4139,7 +4142,7 @@
         <v>45.0</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I67" s="1">
         <v>22.5</v>
@@ -4175,7 +4178,7 @@
         <v>3.0</v>
       </c>
       <c r="T67" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="68">
@@ -4189,7 +4192,7 @@
         <v>50.0</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I68" s="1">
         <v>25.0</v>
@@ -4225,7 +4228,7 @@
         <v>3.0</v>
       </c>
       <c r="T68" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="69">
@@ -4233,7 +4236,7 @@
         <v>95</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F69" s="1">
         <v>8.0</v>
@@ -4242,7 +4245,7 @@
         <v>0.0</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I69" s="1">
         <v>5.0</v>
@@ -4278,12 +4281,12 @@
         <v>18.0</v>
       </c>
       <c r="T69" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="70">
       <c r="E70" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F70" s="1">
         <v>8.0</v>
@@ -4292,7 +4295,7 @@
         <v>10.0</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I70" s="1">
         <v>10.0</v>
@@ -4328,7 +4331,7 @@
         <v>18.0</v>
       </c>
       <c r="T70" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="71">
@@ -4342,7 +4345,7 @@
         <v>15.0</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I71" s="1">
         <v>7.5</v>
@@ -4378,7 +4381,7 @@
         <v>18.0</v>
       </c>
       <c r="T71" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="72">
@@ -4392,7 +4395,7 @@
         <v>20.0</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I72" s="1">
         <v>10.0</v>
@@ -4428,7 +4431,7 @@
         <v>18.0</v>
       </c>
       <c r="T72" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="73">
@@ -4442,7 +4445,7 @@
         <v>25.0</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I73" s="1">
         <v>12.5</v>
@@ -4478,7 +4481,7 @@
         <v>18.0</v>
       </c>
       <c r="T73" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="74">
@@ -4492,7 +4495,7 @@
         <v>30.0</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I74" s="1">
         <v>15.0</v>
@@ -4528,7 +4531,7 @@
         <v>18.0</v>
       </c>
       <c r="T74" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="75">
@@ -4542,7 +4545,7 @@
         <v>35.0</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I75" s="1">
         <v>17.5</v>
@@ -4578,7 +4581,7 @@
         <v>18.0</v>
       </c>
       <c r="T75" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="76">
@@ -4592,7 +4595,7 @@
         <v>40.0</v>
       </c>
       <c r="H76" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I76" s="1">
         <v>20.0</v>
@@ -4628,7 +4631,7 @@
         <v>18.0</v>
       </c>
       <c r="T76" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="77">
@@ -4642,7 +4645,7 @@
         <v>45.0</v>
       </c>
       <c r="H77" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I77" s="1">
         <v>22.5</v>
@@ -4678,7 +4681,7 @@
         <v>18.0</v>
       </c>
       <c r="T77" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="78">
@@ -4692,7 +4695,7 @@
         <v>50.0</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I78" s="1">
         <v>25.0</v>
@@ -4728,7 +4731,520 @@
         <v>18.0</v>
       </c>
       <c r="T78" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F79" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G79" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I79" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="J79" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="K79" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L79" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="M79" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N79" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O79" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P79" s="1">
+        <f t="shared" ref="P79:P88" si="6">4*12</f>
+        <v>48</v>
+      </c>
+      <c r="Q79" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R79" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S79" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T79" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="E80" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F80" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G80" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I80" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="J80" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="K80" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L80" s="1">
+        <v>32.0</v>
+      </c>
+      <c r="M80" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N80" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="O80" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P80" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q80" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R80" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S80" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T80" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="E81" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F81" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G81" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I81" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="J81" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="K81" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L81" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="M81" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N81" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O81" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P81" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q81" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R81" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S81" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T81" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="E82" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F82" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G82" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I82" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="J82" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="K82" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L82" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="M82" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N82" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O82" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P82" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q82" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R82" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S82" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T82" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="E83" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F83" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G83" s="1">
+        <v>25.0</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I83" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="J83" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="K83" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L83" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="M83" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N83" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O83" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P83" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q83" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R83" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S83" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T83" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="E84" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F84" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G84" s="1">
+        <v>30.0</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I84" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="J84" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="K84" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L84" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="M84" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N84" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O84" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P84" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q84" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R84" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S84" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T84" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="E85" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F85" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G85" s="1">
+        <v>35.0</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I85" s="1">
+        <v>17.5</v>
+      </c>
+      <c r="J85" s="1">
+        <v>17.5</v>
+      </c>
+      <c r="K85" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L85" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="M85" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N85" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O85" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P85" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q85" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R85" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S85" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T85" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="E86" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F86" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G86" s="1">
+        <v>40.0</v>
+      </c>
+      <c r="H86" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I86" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="J86" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="K86" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L86" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="M86" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N86" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O86" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P86" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q86" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R86" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S86" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T86" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="E87" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F87" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="G87" s="1">
+        <v>45.0</v>
+      </c>
+      <c r="H87" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I87" s="1">
+        <v>22.5</v>
+      </c>
+      <c r="J87" s="1">
+        <v>22.5</v>
+      </c>
+      <c r="K87" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L87" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="M87" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N87" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O87" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P87" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q87" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R87" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S87" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T87" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="E88" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F88" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G88" s="1">
+        <v>50.0</v>
+      </c>
+      <c r="H88" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I88" s="1">
+        <v>25.0</v>
+      </c>
+      <c r="J88" s="1">
+        <v>25.0</v>
+      </c>
+      <c r="K88" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="L88" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="M88" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="N88" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="O88" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="P88" s="1">
+        <f t="shared" si="6"/>
+        <v>48</v>
+      </c>
+      <c r="Q88" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="R88" s="1">
+        <v>48.0</v>
+      </c>
+      <c r="S88" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="T88" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -4753,26 +5269,26 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" ht="15.0" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1"/>
@@ -5797,15 +6313,15 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" ht="15.0" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="1">
@@ -5813,20 +6329,20 @@
         <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" ht="15.0" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>29</v>
@@ -5834,31 +6350,31 @@
     </row>
     <row r="6" ht="15.0" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>37</v>
@@ -5866,7 +6382,7 @@
     </row>
     <row r="10" ht="15.0" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>38</v>
@@ -5877,15 +6393,15 @@
         <v>15</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="1">
@@ -5893,7 +6409,7 @@
         <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="1">
@@ -5901,7 +6417,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" ht="15.0" customHeight="1">
@@ -5909,12 +6425,12 @@
         <v>21</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>46</v>
@@ -5922,7 +6438,7 @@
     </row>
     <row r="17" ht="15.0" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>47</v>
@@ -5946,7 +6462,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>52</v>
@@ -5954,26 +6470,26 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1"/>

</xml_diff>